<commit_message>
- set header color in Excel - set default value for minDate
</commit_message>
<xml_diff>
--- a/api/templates/result_counts_by_hiv_status/en.xlsx
+++ b/api/templates/result_counts_by_hiv_status/en.xlsx
@@ -102,7 +102,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39994506668294322"/>
+        <fgColor rgb="FF3CC0DD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -144,13 +144,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -187,6 +187,11 @@
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FF3CC0DD"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -510,33 +515,33 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="13" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="13"/>
+      <c r="E5" s="11"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>

</xml_diff>